<commit_message>
Updated Python Excel File
</commit_message>
<xml_diff>
--- a/CAP776.xlsx
+++ b/CAP776.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="86">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -280,6 +280,12 @@
   </si>
   <si>
     <t>Tired.</t>
+  </si>
+  <si>
+    <t>Take proper sleep and do the tasks related to core subjects.</t>
+  </si>
+  <si>
+    <t>Learning skills.</t>
   </si>
 </sst>
 </file>
@@ -1564,9 +1570,10 @@
   <dimension ref="A1:N401"/>
   <sheetFormatPr defaultColWidth="8.57407407407407" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="14.7777777777778" customWidth="1"/>
+    <col min="1" max="1" width="10.3240740740741" customWidth="1"/>
     <col min="2" max="2" width="10.8888888888889" customWidth="1"/>
-    <col min="3" max="6" width="11" customWidth="1"/>
+    <col min="3" max="3" width="11.5555555555556" customWidth="1"/>
+    <col min="4" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="13" customWidth="1"/>
     <col min="8" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
@@ -2936,11 +2943,11 @@
       <c r="A33" s="8">
         <v>46274</v>
       </c>
-      <c r="B33" s="8">
-        <v>46275</v>
-      </c>
-      <c r="C33" s="8">
-        <v>46276</v>
+      <c r="B33" s="9">
+        <v>300</v>
+      </c>
+      <c r="C33" s="9">
+        <v>60</v>
       </c>
       <c r="D33" s="9">
         <v>120</v>
@@ -2959,11 +2966,11 @@
       </c>
       <c r="I33" s="13">
         <f t="shared" si="0"/>
-        <v>93051</v>
+        <v>860</v>
       </c>
       <c r="J33" s="13">
         <f t="shared" si="1"/>
-        <v>-91611</v>
+        <v>580</v>
       </c>
       <c r="K33" s="14" t="s">
         <v>57</v>
@@ -2982,11 +2989,11 @@
       <c r="A34" s="8">
         <v>46275</v>
       </c>
-      <c r="B34" s="8">
-        <v>46276</v>
-      </c>
-      <c r="C34" s="8">
-        <v>46277</v>
+      <c r="B34" s="9">
+        <v>420</v>
+      </c>
+      <c r="C34" s="9">
+        <v>60</v>
       </c>
       <c r="D34" s="9">
         <v>180</v>
@@ -3005,11 +3012,11 @@
       </c>
       <c r="I34" s="13">
         <f t="shared" si="0"/>
-        <v>93263</v>
+        <v>1190</v>
       </c>
       <c r="J34" s="13">
         <f t="shared" si="1"/>
-        <v>-91823</v>
+        <v>250</v>
       </c>
       <c r="K34" s="14" t="s">
         <v>56</v>
@@ -3028,11 +3035,11 @@
       <c r="A35" s="8">
         <v>46276</v>
       </c>
-      <c r="B35" s="8">
-        <v>46277</v>
-      </c>
-      <c r="C35" s="8">
-        <v>46278</v>
+      <c r="B35" s="9">
+        <v>480</v>
+      </c>
+      <c r="C35" s="9">
+        <v>60</v>
       </c>
       <c r="D35" s="9">
         <v>120</v>
@@ -3051,11 +3058,11 @@
       </c>
       <c r="I35" s="13">
         <f t="shared" si="0"/>
-        <v>93155</v>
+        <v>1140</v>
       </c>
       <c r="J35" s="13">
         <f t="shared" si="1"/>
-        <v>-91715</v>
+        <v>300</v>
       </c>
       <c r="K35" s="14" t="s">
         <v>57</v>
@@ -3070,49 +3077,97 @@
         <v>74</v>
       </c>
     </row>
-    <row r="36" spans="1:14">
-      <c r="A36" s="8"/>
-      <c r="B36" s="9"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="9"/>
-      <c r="H36" s="9"/>
-      <c r="I36" s="13" t="str">
+    <row r="36" ht="28.8" spans="1:14">
+      <c r="A36" s="8">
+        <v>46277</v>
+      </c>
+      <c r="B36" s="9">
+        <v>480</v>
+      </c>
+      <c r="C36" s="9">
+        <v>0</v>
+      </c>
+      <c r="D36" s="9">
+        <v>180</v>
+      </c>
+      <c r="E36" s="9">
+        <v>60</v>
+      </c>
+      <c r="F36" s="9">
+        <v>0</v>
+      </c>
+      <c r="G36" s="9">
+        <v>0</v>
+      </c>
+      <c r="H36" s="9">
+        <v>180</v>
+      </c>
+      <c r="I36" s="13">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J36" s="13" t="str">
+        <v>900</v>
+      </c>
+      <c r="J36" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K36" s="14"/>
-      <c r="L36" s="14"/>
-      <c r="M36" s="14"/>
-      <c r="N36" s="16"/>
+        <v>540</v>
+      </c>
+      <c r="K36" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="L36" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="M36" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="N36" s="16" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="37" spans="1:14">
-      <c r="A37" s="8"/>
-      <c r="B37" s="9"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="G37" s="9"/>
-      <c r="H37" s="9"/>
-      <c r="I37" s="13" t="str">
+      <c r="A37" s="8">
+        <v>46278</v>
+      </c>
+      <c r="B37" s="9">
+        <v>540</v>
+      </c>
+      <c r="C37" s="9">
+        <v>0</v>
+      </c>
+      <c r="D37" s="9">
+        <v>120</v>
+      </c>
+      <c r="E37" s="9">
+        <v>60</v>
+      </c>
+      <c r="F37" s="9">
+        <v>0</v>
+      </c>
+      <c r="G37" s="9">
+        <v>0</v>
+      </c>
+      <c r="H37" s="9">
+        <v>240</v>
+      </c>
+      <c r="I37" s="13">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="13" t="str">
+        <v>960</v>
+      </c>
+      <c r="J37" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="14"/>
-      <c r="L37" s="14"/>
-      <c r="M37" s="14"/>
-      <c r="N37" s="16"/>
+        <v>480</v>
+      </c>
+      <c r="K37" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="L37" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="M37" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="N37" s="16" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="38" spans="1:14">
       <c r="A38" s="8"/>

</xml_diff>

<commit_message>
Updated Pyhton Excel File
</commit_message>
<xml_diff>
--- a/CAP776.xlsx
+++ b/CAP776.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="89">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -292,6 +292,9 @@
   </si>
   <si>
     <t>Tired after atttending the so many classes.</t>
+  </si>
+  <si>
+    <t>Preparing for the upcoming CA.</t>
   </si>
 </sst>
 </file>
@@ -3268,48 +3271,96 @@
       </c>
     </row>
     <row r="40" spans="1:14">
-      <c r="A40" s="8"/>
-      <c r="B40" s="9"/>
-      <c r="C40" s="9"/>
-      <c r="D40" s="9"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="9"/>
-      <c r="G40" s="9"/>
-      <c r="H40" s="9"/>
-      <c r="I40" s="13" t="str">
+      <c r="A40" s="8">
+        <v>46281</v>
+      </c>
+      <c r="B40" s="9">
+        <v>300</v>
+      </c>
+      <c r="C40" s="9">
+        <v>60</v>
+      </c>
+      <c r="D40" s="9">
+        <v>120</v>
+      </c>
+      <c r="E40" s="9">
+        <v>60</v>
+      </c>
+      <c r="F40" s="9">
+        <v>200</v>
+      </c>
+      <c r="G40" s="9">
+        <v>4</v>
+      </c>
+      <c r="H40" s="9">
+        <v>240</v>
+      </c>
+      <c r="I40" s="13">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J40" s="13" t="str">
+        <v>980</v>
+      </c>
+      <c r="J40" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K40" s="14"/>
-      <c r="L40" s="14"/>
-      <c r="M40" s="14"/>
-      <c r="N40" s="16"/>
+        <v>460</v>
+      </c>
+      <c r="K40" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="L40" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="M40" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="N40" s="16" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="41" spans="1:14">
-      <c r="A41" s="8"/>
-      <c r="B41" s="9"/>
-      <c r="C41" s="9"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="9"/>
-      <c r="F41" s="9"/>
-      <c r="G41" s="9"/>
-      <c r="H41" s="9"/>
-      <c r="I41" s="13" t="str">
+      <c r="A41" s="8">
+        <v>46282</v>
+      </c>
+      <c r="B41" s="9">
+        <v>480</v>
+      </c>
+      <c r="C41" s="9">
+        <v>60</v>
+      </c>
+      <c r="D41" s="9">
+        <v>60</v>
+      </c>
+      <c r="E41" s="9">
+        <v>0</v>
+      </c>
+      <c r="F41" s="9">
+        <v>350</v>
+      </c>
+      <c r="G41" s="9">
+        <v>7</v>
+      </c>
+      <c r="H41" s="9">
+        <v>240</v>
+      </c>
+      <c r="I41" s="13">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J41" s="13" t="str">
+        <v>1190</v>
+      </c>
+      <c r="J41" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K41" s="14"/>
-      <c r="L41" s="14"/>
-      <c r="M41" s="14"/>
-      <c r="N41" s="16"/>
+        <v>250</v>
+      </c>
+      <c r="K41" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="L41" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="M41" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="N41" s="16" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="42" spans="1:14">
       <c r="A42" s="8"/>

</xml_diff>